<commit_message>
add encoder reset buttons
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kok/CLionProjects/stm32-digital-potentiometer-v2/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FF1EC78-A0CD-8C47-A2AE-4EDECB6935A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80370BDC-76CA-BE4A-8012-4FCFF907EFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{B0D79F4F-D64C-8947-A2F8-5FC1821B31EC}"/>
   </bookViews>
@@ -146,12 +146,6 @@
     <t>01X02 Pin Header</t>
   </si>
   <si>
-    <t>01X03 Pin Header</t>
-  </si>
-  <si>
-    <t>C5383112</t>
-  </si>
-  <si>
     <t>Plugin,P=2.54mm</t>
   </si>
   <si>
@@ -287,9 +281,6 @@
     <t>2541WV-02P</t>
   </si>
   <si>
-    <t>2541WV-03P</t>
-  </si>
-  <si>
     <t>2541WV-04P</t>
   </si>
   <si>
@@ -411,6 +402,15 @@
   </si>
   <si>
     <t>J7</t>
+  </si>
+  <si>
+    <t>01X05Pin Header</t>
+  </si>
+  <si>
+    <t>2541WV-05P</t>
+  </si>
+  <si>
+    <t>C5383114</t>
   </si>
 </sst>
 </file>
@@ -899,49 +899,49 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I1" s="8" t="s">
         <v>2</v>
       </c>
       <c r="K1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="N1" s="8" t="s">
         <v>71</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>73</v>
       </c>
       <c r="O1" s="8" t="s">
         <v>2</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -952,7 +952,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>5</v>
@@ -967,7 +967,7 @@
         <v>1.48</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I2" s="9">
         <f>F2*G2</f>
@@ -1000,10 +1000,10 @@
         <v>13</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>6</v>
@@ -1018,7 +1018,7 @@
         <v>4.8099999999999996</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I3" s="9">
         <f t="shared" ref="I3:I26" si="0">F3*G3</f>
@@ -1030,16 +1030,16 @@
         <v>21</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F4" s="16">
         <v>8</v>
@@ -1048,7 +1048,7 @@
         <v>0.01</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I4" s="9">
         <f t="shared" si="0"/>
@@ -1060,16 +1060,16 @@
         <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D5" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>96</v>
       </c>
       <c r="F5" s="16">
         <v>3</v>
@@ -1078,7 +1078,7 @@
         <v>0.01</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" si="0"/>
@@ -1090,10 +1090,10 @@
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>8</v>
@@ -1108,7 +1108,7 @@
         <v>0.11</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I6" s="9">
         <f t="shared" si="0"/>
@@ -1120,10 +1120,10 @@
         <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>10</v>
@@ -1138,7 +1138,7 @@
         <v>0.08</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I7" s="9">
         <f t="shared" si="0"/>
@@ -1150,16 +1150,16 @@
         <v>14</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F8" s="16">
         <v>12</v>
@@ -1168,7 +1168,7 @@
         <v>0.01</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I8" s="9">
         <f t="shared" si="0"/>
@@ -1180,16 +1180,16 @@
         <v>15</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F9" s="16">
         <v>1</v>
@@ -1198,7 +1198,7 @@
         <v>0.01</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I9" s="9">
         <f t="shared" si="0"/>
@@ -1207,19 +1207,19 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F10" s="16">
         <v>1</v>
@@ -1228,7 +1228,7 @@
         <v>0.04</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I10" s="9">
         <f t="shared" si="0"/>
@@ -1237,19 +1237,19 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F11" s="16">
         <v>1</v>
@@ -1258,7 +1258,7 @@
         <v>0.01</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I11" s="9">
         <f t="shared" si="0"/>
@@ -1267,19 +1267,19 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F12" s="16">
         <v>3</v>
@@ -1288,7 +1288,7 @@
         <v>0.01</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I12" s="9">
         <f t="shared" si="0"/>
@@ -1300,16 +1300,16 @@
         <v>16</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F13" s="16">
         <v>1</v>
@@ -1318,7 +1318,7 @@
         <v>0.01</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I13" s="9">
         <f t="shared" si="0"/>
@@ -1330,10 +1330,10 @@
         <v>19</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>18</v>
@@ -1348,7 +1348,7 @@
         <v>1.65</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I14" s="9">
         <f t="shared" si="0"/>
@@ -1357,19 +1357,19 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F15" s="16">
         <v>2</v>
@@ -1378,7 +1378,7 @@
         <v>0.01</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I15" s="9">
         <f t="shared" si="0"/>
@@ -1390,16 +1390,16 @@
         <v>34</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F16" s="16">
         <v>4</v>
@@ -1408,7 +1408,7 @@
         <v>0.01</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I16" s="9">
         <f t="shared" si="0"/>
@@ -1420,10 +1420,10 @@
         <v>22</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>24</v>
@@ -1438,7 +1438,7 @@
         <v>0.01</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I17" s="9">
         <f t="shared" si="0"/>
@@ -1450,16 +1450,16 @@
         <v>25</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F18" s="16">
         <v>2</v>
@@ -1468,7 +1468,7 @@
         <v>0.01</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I18" s="9">
         <f t="shared" si="0"/>
@@ -1480,10 +1480,10 @@
         <v>28</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>27</v>
@@ -1498,7 +1498,7 @@
         <v>0.17</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" si="0"/>
@@ -1510,16 +1510,16 @@
         <v>35</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D20" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="F20" s="16">
         <v>2</v>
@@ -1528,7 +1528,7 @@
         <v>0.01</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I20" s="9">
         <f t="shared" si="0"/>
@@ -1537,19 +1537,19 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>38</v>
-      </c>
       <c r="E21" s="4" t="s">
-        <v>37</v>
+        <v>124</v>
       </c>
       <c r="F21" s="16">
         <v>2</v>
@@ -1558,7 +1558,7 @@
         <v>0.01</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I21" s="9">
         <f t="shared" si="0"/>
@@ -1570,16 +1570,16 @@
         <v>29</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F22" s="16">
         <v>1</v>
@@ -1588,7 +1588,7 @@
         <v>0.01</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I22" s="9">
         <f t="shared" si="0"/>
@@ -1597,19 +1597,19 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>120</v>
-      </c>
       <c r="D23" s="11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F23" s="16">
         <v>2</v>
@@ -1618,7 +1618,7 @@
         <v>0.02</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" si="0"/>
@@ -1627,19 +1627,19 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>31</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F24" s="16">
         <v>1</v>
@@ -1648,7 +1648,7 @@
         <v>0.02</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I24" s="9">
         <f t="shared" si="0"/>
@@ -1657,19 +1657,19 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>124</v>
-      </c>
       <c r="D25" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F25" s="16">
         <v>1</v>
@@ -1678,7 +1678,7 @@
         <v>0.16</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I25" s="9">
         <f t="shared" si="0"/>
@@ -1690,10 +1690,10 @@
         <v>32</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>31</v>
@@ -1708,7 +1708,7 @@
         <v>0.03</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I26" s="9">
         <f t="shared" si="0"/>

</xml_diff>